<commit_message>
Day 2: Tax agent, Excel migration, wealth restructure
- Migrate portfolio data layer to Excel (.xlsx per category)
- Add employee-equity.xlsx and angel-investment.xlsx, remove startups.xlsx
- Restructure wealth view with category detail pages and sidebar nav
- Build Tax page: overview stats, asset location analysis, hidden liability, taxable events
- Add info tooltips for tax treatment groups (reuse profile pattern)
- Fix tax rate consistency (profile.json as source of truth, not tax-summary.json)
- Fix 529 missing from hidden liability tax-free calculation
- Add capis-tax independent agent (.claude/agents/) with web-verified rates and data backfill
- Add tax-professional reference skill
- Document agent architecture and data backfill convention in CLAUDE.md
- Update DEVLOG with Day 2 progress and blockers

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/art.xlsx
+++ b/data/art.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:L2"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -405,19 +405,12 @@
     <col min="4" max="4" width="10.83203125" customWidth="1"/>
     <col min="5" max="5" width="12.83203125" customWidth="1"/>
     <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" customWidth="1"/>
-    <col min="8" max="8" width="50.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="22.83203125" customWidth="1"/>
+    <col min="7" max="7" width="50.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="22.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
     <col min="11" max="11" width="12.83203125" customWidth="1"/>
     <col min="12" max="12" width="12.83203125" customWidth="1"/>
-    <col min="13" max="13" width="10.83203125" customWidth="1"/>
-    <col min="14" max="14" width="10.83203125" customWidth="1"/>
-    <col min="15" max="15" width="10.83203125" customWidth="1"/>
-    <col min="16" max="16" width="10.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="10.83203125" customWidth="1"/>
-    <col min="19" max="19" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -440,43 +433,22 @@
         <v>currentPrice</v>
       </c>
       <c r="G1" t="str">
-        <v>change24h</v>
+        <v>notes</v>
       </c>
       <c r="H1" t="str">
-        <v>notes</v>
+        <v>accountType</v>
       </c>
       <c r="I1" t="str">
-        <v>accountType</v>
+        <v>accountName</v>
       </c>
       <c r="J1" t="str">
-        <v>accountName</v>
+        <v>costBasis</v>
       </c>
       <c r="K1" t="str">
-        <v>costBasis</v>
+        <v>purchaseDate</v>
       </c>
       <c r="L1" t="str">
-        <v>purchaseDate</v>
-      </c>
-      <c r="M1" t="str">
-        <v>Day 1</v>
-      </c>
-      <c r="N1" t="str">
-        <v>Day 2</v>
-      </c>
-      <c r="O1" t="str">
-        <v>Day 3</v>
-      </c>
-      <c r="P1" t="str">
-        <v>Day 4</v>
-      </c>
-      <c r="Q1" t="str">
-        <v>Day 5</v>
-      </c>
-      <c r="R1" t="str">
-        <v>Day 6</v>
-      </c>
-      <c r="S1" t="str">
-        <v>Day 7</v>
+        <v>lastUpdated</v>
       </c>
     </row>
     <row r="2">
@@ -498,49 +470,28 @@
       <c r="F2">
         <v>4800</v>
       </c>
-      <c r="G2">
-        <v>0</v>
+      <c r="G2" t="str">
+        <v>Open Edition. Secondary market value.</v>
       </c>
       <c r="H2" t="str">
-        <v>Open Edition. Secondary market value.</v>
+        <v>direct</v>
       </c>
       <c r="I2" t="str">
-        <v>direct</v>
-      </c>
-      <c r="J2" t="str">
         <v>Personal Property</v>
       </c>
-      <c r="K2">
+      <c r="J2">
         <v>3200</v>
       </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
       <c r="L2" t="str">
-        <v/>
-      </c>
-      <c r="M2">
-        <v>4800</v>
-      </c>
-      <c r="N2">
-        <v>4800</v>
-      </c>
-      <c r="O2">
-        <v>4800</v>
-      </c>
-      <c r="P2">
-        <v>4800</v>
-      </c>
-      <c r="Q2">
-        <v>4800</v>
-      </c>
-      <c r="R2">
-        <v>4800</v>
-      </c>
-      <c r="S2">
-        <v>4800</v>
+        <v>2026-02-11</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>